<commit_message>
fix(ayuda-memoria): carga OD faltantes (4, 5, 113-ANEXO) y saca la 275/26 ya aprobada
Mariano detectó a mano OD que nunca habían entrado a Ayuda Memoria pese a
estar publicadas (ordenes_dia_2026.xlsx no las traía) y pidió sacar la
275/26 porque ya fue aprobada. Mergeado el xlsx que subió con el existente
(upsert por número/período/tipo) y regenerada Ayuda Memoria.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I102"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1350,7 +1350,7 @@
         <v>2026</v>
       </c>
       <c r="B25" t="n">
-        <v>275</v>
+        <v>321</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1359,13 +1359,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>S-252/26-PL
-S-308/26-PL</t>
+          <t>S-1841/25-PD</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MENDOZA Y OTROS: PROYECTO DE LEY QUE DECLARA HEROE NACIONAL A DON BERNABE ARAOZ.</t>
+          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE RINDE HOMENAJE Y RECONOCE A LOS 68 TRIPULANTES Y PASAJEROS DEL AVIÓN DOUGLAS C-54, DE LA FUERZA AEREA ARGENTINA, EN EL 60 ANIVERSARIO DE SU DESAPARICION EL 3 DE NOVIEMBRE DE 2025.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1389,7 +1388,7 @@
         <v>2026</v>
       </c>
       <c r="B26" t="n">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1398,17 +1397,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>S-1841/25-PD</t>
+          <t>S-1059/25-PD</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE RINDE HOMENAJE Y RECONOCE A LOS 68 TRIPULANTES Y PASAJEROS DEL AVIÓN DOUGLAS C-54, DE LA FUERZA AEREA ARGENTINA, EN EL 60 ANIVERSARIO DE SU DESAPARICION EL 3 DE NOVIEMBRE DE 2025.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LAS "CHARLAS ANTARTICAS", QUE REALIZA LA BIBLIOTECA POPULAR 2 DE ABRIL, DE LA CDAD. DE POSADAS, PROV. DE MISIONES.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>DE DEFENSA NACIONAL -</t>
+          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1427,7 +1426,7 @@
         <v>2026</v>
       </c>
       <c r="B27" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1436,17 +1435,18 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>S-1059/25-PD</t>
+          <t>S-1879/25-PD
+S-457/26-PD</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LAS "CHARLAS ANTARTICAS", QUE REALIZA LA BIBLIOTECA POPULAR 2 DE ABRIL, DE LA CDAD. DE POSADAS, PROV. DE MISIONES.</t>
+          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA CELEBRACIÓN DE LOS CINCUENTA AÑOS DE LA FERIA INTERNACIONAL DEL LIBRO DE BUENOS AIRES, A REALIZARSE EN LA RURAL, DEL 23 DE ABRIL AL 11 DE MAYO DE 2026.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1465,7 +1465,7 @@
         <v>2026</v>
       </c>
       <c r="B28" t="n">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1474,13 +1474,13 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>S-1879/25-PD
-S-457/26-PD</t>
+          <t>S-2136/25-PD
+S-2178/25-PD</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA CELEBRACIÓN DE LOS CINCUENTA AÑOS DE LA FERIA INTERNACIONAL DEL LIBRO DE BUENOS AIRES, A REALIZARSE EN LA RURAL, DEL 23 DE ABRIL AL 11 DE MAYO DE 2026.</t>
+          <t>CAPITANICH: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCIMIENTO A GLORIA ARGENTINA CISNEROS, DOCENTE DE LA PROV. DEL CHACO, POR SU SELECCIÓN COMO FINALISTA DEL GLOBAL TEACHER PRIZE 2026.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1504,7 +1504,7 @@
         <v>2026</v>
       </c>
       <c r="B29" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1513,13 +1513,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>S-2136/25-PD
-S-2178/25-PD</t>
+          <t>S-29/26-PD</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CAPITANICH: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCIMIENTO A GLORIA ARGENTINA CISNEROS, DOCENTE DE LA PROV. DEL CHACO, POR SU SELECCIÓN COMO FINALISTA DEL GLOBAL TEACHER PRIZE 2026.</t>
+          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR LA LABOR DEL EQUIPO RIOJANO, GANADOR EN EL PROGRAMA FEDERAL DE FORMACION "GESTION PARA EL DESARROLLO".</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1543,7 +1542,7 @@
         <v>2026</v>
       </c>
       <c r="B30" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1552,12 +1551,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>S-29/26-PD</t>
+          <t>S-92/26-PD</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR LA LABOR DEL EQUIPO RIOJANO, GANADOR EN EL PROGRAMA FEDERAL DE FORMACION "GESTION PARA EL DESARROLLO".</t>
+          <t>MENDOZA: PROYECTO DE DECLARACIÓN QUE ADHIERE AL ANIVERSARIO DE LA BATALLA DE TUCUMAN, EL 24 DE SEPTIEMBRE DE 2026, RINDIENDO DISTINTOS HOMENAJES AFINES Y EXPRESA RECONOCIMIENTO A LA FESTIVIDAD DE NUESTRA SEÑORA DE LA MERCED.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1581,7 +1580,7 @@
         <v>2026</v>
       </c>
       <c r="B31" t="n">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1590,12 +1589,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>S-92/26-PD</t>
+          <t>S-115/26-PD</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>MENDOZA: PROYECTO DE DECLARACIÓN QUE ADHIERE AL ANIVERSARIO DE LA BATALLA DE TUCUMAN, EL 24 DE SEPTIEMBRE DE 2026, RINDIENDO DISTINTOS HOMENAJES AFINES Y EXPRESA RECONOCIMIENTO A LA FESTIVIDAD DE NUESTRA SEÑORA DE LA MERCED.</t>
+          <t>VALENZUELA Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PRIMER "MUNDIAL DE LA YERBA MATE", A REALIZARSE EN EL MUSEO DEL MATE, CABA, DEL 5 AL 7 DE JUNIO DE 2026.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1619,7 +1618,7 @@
         <v>2026</v>
       </c>
       <c r="B32" t="n">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1628,12 +1627,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>S-115/26-PD</t>
+          <t>S-214/26-PD</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>VALENZUELA Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PRIMER "MUNDIAL DE LA YERBA MATE", A REALIZARSE EN EL MUSEO DEL MATE, CABA, DEL 5 AL 7 DE JUNIO DE 2026.</t>
+          <t>ALMEIDA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA LABOR EDUCATIVA, TECNOLOGICA Y DE INNOVACION DESARROLLADA POR LA ESCUELA PRODIGY, CON SEDES EN DIVERSAS LOCALIDADES DE LAS PROVINCIAS DE RIO NEGRO Y NEUQUEN.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1657,7 +1656,7 @@
         <v>2026</v>
       </c>
       <c r="B33" t="n">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1666,12 +1665,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>S-214/26-PD</t>
+          <t>S-413/26-PD</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ALMEIDA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA LABOR EDUCATIVA, TECNOLOGICA Y DE INNOVACION DESARROLLADA POR LA ESCUELA PRODIGY, CON SEDES EN DIVERSAS LOCALIDADES DE LAS PROVINCIAS DE RIO NEGRO Y NEUQUEN.</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA PUBLICACIÓN Y PRESENTACIÓN DEL LIBRO DE INVESTIGACIÓN "ZAMBA DE MI ESPERANZA. LA QUE SABEMOS TODOS", DE ROBERTO MERCADO.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1695,7 +1694,7 @@
         <v>2026</v>
       </c>
       <c r="B34" t="n">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1704,12 +1703,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>S-413/26-PD</t>
+          <t>S-429/26-PD</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA PUBLICACIÓN Y PRESENTACIÓN DEL LIBRO DE INVESTIGACIÓN "ZAMBA DE MI ESPERANZA. LA QUE SABEMOS TODOS", DE ROBERTO MERCADO.</t>
+          <t>GUZMÁN CORAITA: PROYECTO DE DECLARACIÓN QUE EXPRESA PESAR POR EL FALLECIMIENTO DEL HISTORIADOR ROSARINO MIGUEL ANGEL DE MARCO.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1733,7 +1732,7 @@
         <v>2026</v>
       </c>
       <c r="B35" t="n">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1742,12 +1741,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>S-429/26-PD</t>
+          <t>S-492/26-PD</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>GUZMÁN CORAITA: PROYECTO DE DECLARACIÓN QUE EXPRESA PESAR POR EL FALLECIMIENTO DEL HISTORIADOR ROSARINO MIGUEL ANGEL DE MARCO.</t>
+          <t>CARAMBIA Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL LIBRO "A ORILLAS DEL RIO FENIX" DE LOS AUTORES GRACIELA CISELLI Y MARCELO HERNANDEZ.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1771,7 +1770,7 @@
         <v>2026</v>
       </c>
       <c r="B36" t="n">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1780,12 +1779,13 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>S-492/26-PD</t>
+          <t>S-535/26-PD
+S-613/26-PD</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>CARAMBIA Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL LIBRO "A ORILLAS DEL RIO FENIX" DE LOS AUTORES GRACIELA CISELLI Y MARCELO HERNANDEZ.</t>
+          <t>COTO: PROYECTO DE DECLARACION QUE ADHIERE AL 75° ANIVERSARIO DE LA CREACIÓN DEL INSTITUTO ANTARTICO ARGENTINO, EL 17 DE ABRIL DE 2026.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1809,7 +1809,7 @@
         <v>2026</v>
       </c>
       <c r="B37" t="n">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1818,13 +1818,13 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>S-535/26-PD
-S-613/26-PD</t>
+          <t>S-560/26-PD
+S-623/26-CO</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>COTO: PROYECTO DE DECLARACION QUE ADHIERE AL 75° ANIVERSARIO DE LA CREACIÓN DEL INSTITUTO ANTARTICO ARGENTINO, EL 17 DE ABRIL DE 2026.</t>
+          <t>MOISES: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 70° ANIVERSARIO DE LA ESCUELA NORMAL "GRAL. JOSE DE SAN MARTIN", EN LA CDAD. DE SAN PEDRO DE JUJUY, PROV. DE JUJUY, EL 14 DE MAYO DE 2026.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1848,7 +1848,7 @@
         <v>2026</v>
       </c>
       <c r="B38" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1857,13 +1857,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>S-560/26-PD
-S-623/26-CO</t>
+          <t>S-575/26-PD</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MOISES: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 70° ANIVERSARIO DE LA ESCUELA NORMAL "GRAL. JOSE DE SAN MARTIN", EN LA CDAD. DE SAN PEDRO DE JUJUY, PROV. DE JUJUY, EL 14 DE MAYO DE 2026.</t>
+          <t>BEDIA: PROYECTO DE DECLARACIÓN QUE EXPRESA PESAR POR EL FALLECIMIENTO DEL ACTOR LUIS BRANDONI, EL 20 DE ABRIL DE 2026.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1887,7 +1886,7 @@
         <v>2026</v>
       </c>
       <c r="B39" t="n">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1896,12 +1895,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>S-575/26-PD</t>
+          <t>S-612/26-PD</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BEDIA: PROYECTO DE DECLARACIÓN QUE EXPRESA PESAR POR EL FALLECIMIENTO DEL ACTOR LUIS BRANDONI, EL 20 DE ABRIL DE 2026.</t>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS LA MUESTRA CULTURAL E HISTORICA "CORRIENTES EN CASA ROSADA", A INAUGURARSE EN EL MUSEO DE LA CASA ROSADA,  EN CABA, EL 13 DE MAYO DE 2026.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1925,7 +1924,7 @@
         <v>2026</v>
       </c>
       <c r="B40" t="n">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1934,12 +1933,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>S-612/26-PD</t>
+          <t>S-620/26-PD</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS LA MUESTRA CULTURAL E HISTORICA "CORRIENTES EN CASA ROSADA", A INAUGURARSE EN EL MUSEO DE LA CASA ROSADA,  EN CABA, EL 13 DE MAYO DE 2026.</t>
+          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA CONMEMORACION DEL 40° ANIVERSARIO DE LA CONSTITUCION DE LA PROVINCIA DE SALTA, EL 2 DE JUNIO DE 2026.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1963,7 +1962,7 @@
         <v>2026</v>
       </c>
       <c r="B41" t="n">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1972,17 +1971,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>S-620/26-PD</t>
+          <t>S-1144/26-PL</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA CONMEMORACION DEL 40° ANIVERSARIO DE LA CONSTITUCION DE LA PROVINCIA DE SALTA, EL 2 DE JUNIO DE 2026.</t>
+          <t>ATAUCHE: PROYECTO DE LEY QUE DECLARA HEROE NACIONAL POST MORTEM AL GENERAL MANUEL EDUARDO ARIAS, EN RECONOCIMIENTO A SU ACCIONAR EN LAS GUERRAS POR LA INDEPENDENCIA</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE DEFENSA NACIONAL -</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2001,7 +2000,7 @@
         <v>2026</v>
       </c>
       <c r="B42" t="n">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -2010,17 +2009,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>S-1144/26-PL</t>
+          <t>PE-91/26-AC</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ATAUCHE: PROYECTO DE LEY QUE DECLARA HEROE NACIONAL POST MORTEM AL GENERAL MANUEL EDUARDO ARIAS, EN RECONOCIMIENTO A SU ACCIONAR EN LAS GUERRAS POR LA INDEPENDENCIA</t>
+          <t>MENSAJE N° 101/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ DE CAMARA DEL TRIBUNAL ORAL EN LO CRIMINAL Y CORRECCIONAL N°8 DE LA CAPITAL FEDERAL, AL DR. JUAN MANUEL MEJUTO.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>DE DEFENSA NACIONAL -</t>
+          <t>DE ACUERDOS -</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2039,7 +2038,7 @@
         <v>2026</v>
       </c>
       <c r="B43" t="n">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -2048,17 +2047,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>PE-91/26-AC</t>
+          <t>S-361/26-PL</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>MENSAJE N° 101/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ DE CAMARA DEL TRIBUNAL ORAL EN LO CRIMINAL Y CORRECCIONAL N°8 DE LA CAPITAL FEDERAL, AL DR. JUAN MANUEL MEJUTO.</t>
+          <t>GADANO: PROYECTO DE LEY QUE APRUEBA EL CONVENIO DE CREACION DEL PARQUE INTERJURISDICCIONAL MARINO MONTE LEON, ENTRE EL ESTADO NACIONAL Y LA PROVINCIA DE SANTA CRUZ.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>DE ACUERDOS -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE AMBIENTE Y DESARROLLO SUSTENTABLE -</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2073,11 +2072,15 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B44" t="n">
-        <v>339</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>340</t>
+        </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -2086,17 +2089,22 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>S-361/26-PL</t>
+          <t>OV-453/24-CM</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>GADANO: PROYECTO DE LEY QUE APRUEBA EL CONVENIO DE CREACION DEL PARQUE INTERJURISDICCIONAL MARINO MONTE LEON, ENTRE EL ESTADO NACIONAL Y LA PROVINCIA DE SANTA CRUZ.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO OSCAR ENRIQUE MARTIN, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE VICECÓNSUL HONORARIO DE ESPAÑA EN GRAL. PICO  LA PAMPA.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES - DE AMBIENTE Y DESARROLLO SUSTENTABLE -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2111,11 +2119,15 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B45" t="n">
-        <v>340</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>341</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -2124,435 +2136,539 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>OV-453/24-CM</t>
+          <t>OV-452/24-CM</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO OSCAR ENRIQUE MARTIN, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE VICECÓNSUL HONORARIO DE ESPAÑA EN GRAL. PICO  LA PAMPA.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA FLAVIA LORENA SEAGE, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE VICECONSUL HONORARIA DE ESPAÑA EN PUERTO IGUAZU, MISIONES.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>342</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>OV-451/24-CM</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JOSE CARLOS ARCAGNI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE LETONIA, EN  CABA.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>343</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>OV-450/24-CM</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JUAN CARLOS SCHROEDER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE ALEMANIA EN NEUQUEN.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>344</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>OV-357/26-CM</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO, JUAN LUIS GONZALEZ LANDA, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO VICECONSUL HONORARIO DE LOS ESTADOS UNIDOS MEXICANOS, EN LA CIUDAD DE MENDOZA, PROVINCIA HOM</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B46" t="n">
-        <v>341</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>OV-452/24-CM</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA FLAVIA LORENA SEAGE, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE VICECONSUL HONORARIA DE ESPAÑA EN PUERTO IGUAZU, MISIONES.</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>345</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>OV-331/26-CM</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JAVIER JOSE CALVIÑO, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DEMOCRATICA DE TIMOR-LESTE, EN LA CIUDAD DE SAN ISIDRO, PROV.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
         <is>
           <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B47" t="n">
-        <v>342</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>OV-451/24-CM</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JOSE CARLOS ARCAGNI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE LETONIA, EN  CABA.</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>346</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>OV-300/26-CM</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO RODOLFO ERNESTO CAFFARO KRAMER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DEL REINO DE CAMBOYA, EN LA CIUDAD AUTONÓMA DE BUENOS AIRES, CON C</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
         <is>
           <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B48" t="n">
-        <v>343</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>OV-450/24-CM</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JUAN CARLOS SCHROEDER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE ALEMANIA EN NEUQUEN.</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>347</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>OV-234/24-CM</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO RAUL ENRIQUE BURGOS, QUE SOLICITA AUTORIZACION PARA DESEMPEÑARSE COMO VICECONSUL HONORARIO DE ESPAÑA EN LA CDAD. DE SAN SALVADOR DE JUJUY.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>OV-176/24-CM</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO DANIEL AMADO, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE PORTUGAL EN LA CIUDAD DE COMODORO RIVADAVIA, PROV. DEL CHUBUT.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>349</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>OV-175/24-CM</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA CAROLINA PATRICIA KAHR PIRA, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE AUSTRIA EN LA CIUDAD DE MENDOZA.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>OV-74/26-CM</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO GERMAN ENRIQUE BÖTTGER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REP. FEDERAL DE ALEMANIA EN LA CIUDAD DE SAN MIGUEL DE TUCUMAN, CON</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
         <is>
           <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B49" t="n">
-        <v>344</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>OV-357/26-CM</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO, JUAN LUIS GONZALEZ LANDA, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO VICECONSUL HONORARIO DE LOS ESTADOS UNIDOS MEXICANOS, EN LA CIUDAD DE MENDOZA, PROVINCIA HOMONIMA, CON JURISDICCION EN LAS PROVINCIAS DE SAN JUAN Y SAN LUIS.</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>351</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>OV-32/26-CM</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA ORIANA LAURA FOSSATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO AGENTE CÓNSULAR ADJUNTO DEL CONSULADO DE LA REPUBLICA ITALIANA EN MAR DEL PLATA, PROV, DE BS.AS.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
         <is>
           <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B50" t="n">
-        <v>345</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>OV-331/26-CM</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JAVIER JOSE CALVIÑO, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DEMOCRATICA DE TIMOR-LESTE, EN LA CIUDAD DE SAN ISIDRO, PROV. DE BS. AS., CON CIRCUNSCRIPCIÓN CONSULAR EN TODO EL TERRITORIO NACIONAL.</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>OV-31/26-CM</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO : REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JORGE LUIS PEREZ ALATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DE SINGAPUR EN LA CIUDAD AUTONOMA DE BUENOS AIRES.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
         <is>
           <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B51" t="n">
-        <v>346</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>OV-300/26-CM</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO RODOLFO ERNESTO CAFFARO KRAMER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DEL REINO DE CAMBOYA, EN LA CIUDAD AUTONÓMA DE BUENOS AIRES, CON CIRCUNSCRIPCIÓN CONSULAR EN TODO EL TERRITORIO NACIONAL.</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B52" t="n">
-        <v>347</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>OV-234/24-CM</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO RAUL ENRIQUE BURGOS, QUE SOLICITA AUTORIZACION PARA DESEMPEÑARSE COMO VICECONSUL HONORARIO DE ESPAÑA EN LA CDAD. DE SAN SALVADOR DE JUJUY.</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B53" t="n">
-        <v>348</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>OV-176/24-CM</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO DANIEL AMADO, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE PORTUGAL EN LA CIUDAD DE COMODORO RIVADAVIA, PROV. DEL CHUBUT.</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B54" t="n">
-        <v>349</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>OV-175/24-CM</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA CAROLINA PATRICIA KAHR PIRA, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE AUSTRIA EN LA CIUDAD DE MENDOZA.</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B55" t="n">
-        <v>350</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>OV-74/26-CM</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO GERMAN ENRIQUE BÖTTGER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REP. FEDERAL DE ALEMANIA EN LA CIUDAD DE SAN MIGUEL DE TUCUMAN, CON CIRCUNSCRIPCION EN LAS PROVINCIAS DE CATAMARCA, SANTIAGO DEL ESTERO Y TUCUMAN.</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B56" t="n">
-        <v>351</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>OV-32/26-CM</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA ORIANA LAURA FOSSATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO AGENTE CÓNSULAR ADJUNTO DEL CONSULADO DE LA REPUBLICA ITALIANA EN MAR DEL PLATA, PROV, DE BS.AS.</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2571,7 +2687,7 @@
         <v>2026</v>
       </c>
       <c r="B57" t="n">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2580,17 +2696,17 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>OV-31/26-CM</t>
+          <t>PE-35/26-AC</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JORGE LUIS PEREZ ALATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DE SINGAPUR EN LA CIUDAD AUTONOMA DE BUENOS AIRES.</t>
+          <t>MENSAJE N° 46/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA B,  AL DR. ALEJANDRO JAVIER CATANIA.</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+          <t>DE ACUERDOS -</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2609,7 +2725,7 @@
         <v>2026</v>
       </c>
       <c r="B58" t="n">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -2618,12 +2734,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>PE-35/26-AC</t>
+          <t>PE-37/26-AC</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>MENSAJE N° 46/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA B,  AL DR. ALEJANDRO JAVIER CATANIA.</t>
+          <t>MENSAJE N° 48/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA A, AL DR. JUAN PEDRO GALVAN GREENWAY.</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2647,7 +2763,7 @@
         <v>2026</v>
       </c>
       <c r="B59" t="n">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -2656,17 +2772,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PE-37/26-AC</t>
+          <t>S-517/25-PL</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MENSAJE N° 48/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA A, AL DR. JUAN PEDRO GALVAN GREENWAY.</t>
+          <t>DE ANGELI: PROYECTO DE LEY QUE INSTITUYE EL DIA 15 DE ABRIL DE CADA AÑO COMO EL "DIA NACIONAL DEL INMIGRANTE ALEMAN DEL VOLGA".</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>DE ACUERDOS -</t>
+          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2685,7 +2801,7 @@
         <v>2026</v>
       </c>
       <c r="B60" t="n">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -2694,12 +2810,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>S-517/25-PL</t>
+          <t>S-697/25-PL</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>DE ANGELI: PROYECTO DE LEY QUE INSTITUYE EL DIA 15 DE ABRIL DE CADA AÑO COMO EL "DIA NACIONAL DEL INMIGRANTE ALEMAN DEL VOLGA".</t>
+          <t>AVILA: PROYECTO DE LEY QUE INCORPORA EL ART. 4 BIS A SU SIMILAR 25.415- PROGRAMA DE DETECCION DE LA HIPOACUSIA-, RESPECTO DE INCORPORAR DIVERSAS ACCIONES EN EL AMBITO EDUCATIVO.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2723,7 +2839,7 @@
         <v>2026</v>
       </c>
       <c r="B61" t="n">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -2732,12 +2848,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>S-697/25-PL</t>
+          <t>S-319/25-PL</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE INCORPORA EL ART. 4 BIS A SU SIMILAR 25.415- PROGRAMA DE DETECCION DE LA HIPOACUSIA-, RESPECTO DE INCORPORAR DIVERSAS ACCIONES EN EL AMBITO EDUCATIVO.</t>
+          <t>HUALA: REPRODUCE PROYECTO DE LEY QUE INSTITUYE EL 2 DE MAYO DE CADA AÑO COMO "DIA NACIONAL PARA LA PREVENCION DEL BULLYING Y OTRAS FORMAS DE VIOLENCIA Y ACOSO ESCOLAR". (REF. S. 1243/23)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2761,7 +2877,7 @@
         <v>2026</v>
       </c>
       <c r="B62" t="n">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -2770,12 +2886,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>S-319/25-PL</t>
+          <t>S-404/26-PL</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>HUALA: REPRODUCE PROYECTO DE LEY QUE INSTITUYE EL 2 DE MAYO DE CADA AÑO COMO "DIA NACIONAL PARA LA PREVENCION DEL BULLYING Y OTRAS FORMAS DE VIOLENCIA Y ACOSO ESCOLAR". (REF. S. 1243/23)</t>
+          <t>GADANO: PROYECTO DE LEY QUE INSTITUYE EL DIA 27 DE NOVIEMBRE DE CADA AÑO COMO "DIA DEL BASTON VERDE".</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2799,7 +2915,7 @@
         <v>2026</v>
       </c>
       <c r="B63" t="n">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2808,12 +2924,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>S-404/26-PL</t>
+          <t>S-997/26-PL</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>GADANO: PROYECTO DE LEY QUE INSTITUYE EL DIA 27 DE NOVIEMBRE DE CADA AÑO COMO "DIA DEL BASTON VERDE".</t>
+          <t>AVILA: PROYECTO DE LEY QUE ESTABLECE EL TERCER JUEVES DE MARZO DE CADA AÑO COMO EL "DIA DE REFLEXIÓN CONTRA LA VIOLENCIA JUVENIL.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2833,11 +2949,15 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B64" t="n">
-        <v>359</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>360</t>
+        </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2846,17 +2966,22 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>S-997/26-PL</t>
+          <t>PE-243/26-CE</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE ESTABLECE EL TERCER JUEVES DE MARZO DE CADA AÑO COMO EL "DIA DE REFLEXIÓN CONTRA LA VIOLENCIA JUVENIL.</t>
+          <t>JEFATURA DE GABINETE: COMUNICA EL "ACUERDO DE TRANSFERENCIA DE LA FUNCION JUDICIAL EN MATERIA CRIMINAL Y CORRECCIONAL DE MENORES DEL ÁMBITO NACIONAL A LA JUSTICIA DE LA CIUDAD AUTÓNOMA DE BUENOS AIRES", CELEBRADO EL 3 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -2871,11 +2996,15 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B65" t="n">
-        <v>360</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>361</t>
+        </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -2884,17 +3013,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>PE-243/26-CE</t>
+          <t>PE-244/26-CE</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>JEFATURA DE GABINETE: COMUNICA EL "ACUERDO DE TRANSFERENCIA DE LA FUNCION JUDICIAL EN MATERIA CRIMINAL Y CORRECCIONAL DE MENORES DEL ÁMBITO NACIONAL A LA JUSTICIA DE LA CIUDAD AUTÓNOMA DE BUENOS AIRES", CELEBRADO EL 3 DE JULIO DE 2026.</t>
+          <t>JEFATURA DE GABINETE: COMUNICA EL CUARTO CONVENIO DE TRANSFERENCIA PROGRESIVA DE COMPETENCIAS PENALES DE LA JUSTICIA NACIONAL AL PODER JUDICIAL DE LA CIUDAD AUTÓNOMA DE BUENOS AIRES", CELEBRADO EL 3 DE JULIO DE 2026</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2913,52 +3047,14 @@
         <v>2026</v>
       </c>
       <c r="B66" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>ANEXO</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
-        <is>
-          <t>PE-244/26-CE</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>JEFATURA DE GABINETE: COMUNICA EL CUARTO CONVENIO DE TRANSFERENCIA PROGRESIVA DE COMPETENCIAS PENALES DE LA JUSTICIA NACIONAL AL PODER JUDICIAL DE LA CIUDAD AUTÓNOMA DE BUENOS AIRES", CELEBRADO EL 3 DE JULIO DE 2026</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B67" t="n">
-        <v>362</v>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>ANEXO</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
         <is>
           <t>S-1271/25-PL
 S-1861/25-PL
@@ -2969,40 +3065,40 @@
 S-1246/26-PL</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>AVILA: PROYECTO DE LEY QUE MODIFICA SU SIMILAR 27.640 - BIOCOMBUSTIBLES-, RESPECTO DEL PORCENTAJE OBLIGATORIO DE BIODIESEL Y BIOETANOL EN EL GASOIL Y LA NAFTA.</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES -</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B68" t="n">
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B67" t="n">
         <v>362</v>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
         <is>
           <t>S-1271/25-PL
 S-1861/25-PL
@@ -3013,14 +3109,52 @@
 S-1246/26-PL</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>AVILA: PROYECTO DE LEY QUE MODIFICA SU SIMILAR 27.640 - BIOCOMBUSTIBLES-, RESPECTO DEL PORCENTAJE OBLIGATORIO DE BIODIESEL Y BIOETANOL EN EL GASOIL Y LA NAFTA.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES -</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B68" t="n">
+        <v>363</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>CD-21/25-PL</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE MODIFICA SU SIMILAR 27.640 - BIOCOMBUSTIBLES-, RESPECTO DEL PORCENTAJE OBLIGATORIO DE BIODIESEL Y BIOETANOL EN EL GASOIL Y LA NAFTA.</t>
+          <t>PROYECTO DE LEY EN REVISION QUE DECLARA HEROE NACIONAL AL BRIGADIER ESTANISLAO LOPEZ "PATRIARCA DEL FEDERALISMO ARGENTINO" EN RECONOCIMIENTO A SU ACCIONAR EN DEFENSA DE LOS IDEALES FEDERALES Y REPUBLICANOS.</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES -</t>
+          <t>DE DEFENSA NACIONAL - DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3039,7 +3173,7 @@
         <v>2026</v>
       </c>
       <c r="B69" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -3048,17 +3182,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>CD-21/25-PL</t>
+          <t>S-1040/26-PL</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>PROYECTO DE LEY EN REVISION QUE DECLARA HEROE NACIONAL AL BRIGADIER ESTANISLAO LOPEZ "PATRIARCA DEL FEDERALISMO ARGENTINO" EN RECONOCIMIENTO A SU ACCIONAR EN DEFENSA DE LOS IDEALES FEDERALES Y REPUBLICANOS.</t>
+          <t>VALENZUELA: PROYECTO DE LEY QUE DECLARA FIESTA NACIONAL AL "FESTIVAL DEL FOLCLORE CORRENTINO", A REALIZARSE EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, EN EL MES DE DICIEMBRE DE CADA AÑO.</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>DE DEFENSA NACIONAL - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3077,7 +3211,7 @@
         <v>2026</v>
       </c>
       <c r="B70" t="n">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -3086,12 +3220,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>S-1040/26-PL</t>
+          <t>S-1239/26-PL</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE LEY QUE DECLARA FIESTA NACIONAL AL "FESTIVAL DEL FOLCLORE CORRENTINO", A REALIZARSE EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, EN EL MES DE DICIEMBRE DE CADA AÑO.</t>
+          <t>COTO: PROYECTO DE LEY QUE INSTITUYE EL 3 DE MARZO DE CADA AÑO, COMO "DIA NACIONAL EN HONOR AL ALMIRANTE GUILLERMO BROWN".</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3115,7 +3249,7 @@
         <v>2026</v>
       </c>
       <c r="B71" t="n">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -3123,58 +3257,58 @@
         </is>
       </c>
       <c r="D71" t="inlineStr">
-        <is>
-          <t>S-1239/26-PL</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>COTO: PROYECTO DE LEY QUE INSTITUYE EL 3 DE MARZO DE CADA AÑO, COMO "DIA NACIONAL EN HONOR AL ALMIRANTE GUILLERMO BROWN".</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B72" t="n">
-        <v>366</v>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
         <is>
           <t>S-718/26-PL
 S-808/26-PL
 S-865/26-PL</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>CAPITANICH: PROYECTO DE LEY QUE ESTABLECE UN MARCO REGULATORIO PARA LA EMISIÓN Y DESARROLLO DE ACTIVOS FINANCIEROS AMBIENTALES (AFA).</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>DE LEGISLACIÓN GENERAL - DE AMBIENTE Y DESARROLLO SUSTENTABLE - DE PRESUPUESTO Y HACIENDA -</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B72" t="n">
+        <v>367</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>CD-7/26-PL</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>CAPITANICH: PROYECTO DE LEY QUE ESTABLECE UN MARCO REGULATORIO PARA LA EMISIÓN Y DESARROLLO DE ACTIVOS FINANCIEROS AMBIENTALES (AFA).</t>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA CARTA ORGANICA DEL BANCO CENTRAL DE LA REPUBLICA ARGENTINA.</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>DE LEGISLACIÓN GENERAL - DE AMBIENTE Y DESARROLLO SUSTENTABLE - DE PRESUPUESTO Y HACIENDA -</t>
+          <t>DE ECONOMÍA NACIONAL E INVERSIÓN - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3193,7 +3327,7 @@
         <v>2026</v>
       </c>
       <c r="B73" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -3202,17 +3336,17 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>CD-7/26-PL</t>
+          <t>S-1643/25-PL</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA CARTA ORGANICA DEL BANCO CENTRAL DE LA REPUBLICA ARGENTINA.</t>
+          <t>VISCHI: REPRODUCE PROYECTO DE LEY QUE DECLARA BIEN HISTORICO NACIONAL, EN LOS TERMINOS DE LA LEY 12.665 Y S/M., AL INMUEBLE IDENTIFICADO COMO EX "HOTEL DE INMIGRANTES- EX OFICINAS DE PUENTES Y CAMINOS DE GOYA", SITO EN LA MANZANA N° 497, ENTRE LAS CALLES CAÁ GUAZU Y AV. SARMIENTO DE LA CIUDAD DE GOYA, PROV. DE CORRIENTES. (REF. S.1422/22)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>DE ECONOMÍA NACIONAL E INVERSIÓN - DE PRESUPUESTO Y HACIENDA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3231,7 +3365,7 @@
         <v>2026</v>
       </c>
       <c r="B74" t="n">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -3240,12 +3374,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>S-1643/25-PL</t>
+          <t>S-124/26-PL</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>VISCHI: REPRODUCE PROYECTO DE LEY QUE DECLARA BIEN HISTORICO NACIONAL, EN LOS TERMINOS DE LA LEY 12.665 Y S/M., AL INMUEBLE IDENTIFICADO COMO EX "HOTEL DE INMIGRANTES- EX OFICINAS DE PUENTES Y CAMINOS DE GOYA", SITO EN LA MANZANA N° 497, ENTRE LAS CALLES CAÁ GUAZU Y AV. SARMIENTO DE LA CIUDAD DE GOYA, PROV. DE CORRIENTES. (REF. S.1422/22)</t>
+          <t>AVILA: PROYECTO DE LEY QUE DECLARA MONUMENTO HISTORICO NACIONAL AL CEMENTERIO OESTE DE SAN MIGUEL DE TUCUMAN, PROV. DE TUCUMAN.</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3269,7 +3403,7 @@
         <v>2026</v>
       </c>
       <c r="B75" t="n">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -3278,12 +3412,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>S-124/26-PL</t>
+          <t>S-255/26-PL</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE DECLARA MONUMENTO HISTORICO NACIONAL AL CEMENTERIO OESTE DE SAN MIGUEL DE TUCUMAN, PROV. DE TUCUMAN.</t>
+          <t>FAMA: REPRODUCE PROYECTO DE LEY QUE MODIFICA SU SIMILAR 26.206 -EDUCACION NACIONAL-  RESPECTO DE PROMOVER EL DESARROLLO DE LA EDUCACION EMOCIONAL. (REF. S. 752/22)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3307,7 +3441,7 @@
         <v>2026</v>
       </c>
       <c r="B76" t="n">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -3316,12 +3450,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>S-255/26-PL</t>
+          <t>S-447/26-PL</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>FAMA: REPRODUCE PROYECTO DE LEY QUE MODIFICA SU SIMILAR 26.206 -EDUCACION NACIONAL-  RESPECTO DE PROMOVER EL DESARROLLO DE LA EDUCACION EMOCIONAL. (REF. S. 752/22)</t>
+          <t>MENDOZA Y OTROS: REPRODUCE PROYECTO DE LEY QUE DECLARA PATRIMONIO INMATERIAL CULTURAL Y NATURAL DE LA NACION, EN LOS TERMINOS DE LA LEY 26.118, AL "CHAKU", PRACTICA ANCESTRAL INCAICA DE CAPTURA, ESQUILA Y LIBERACIÓN DE VICUÑAS. (REF. S. 830/24).</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3345,7 +3479,7 @@
         <v>2026</v>
       </c>
       <c r="B77" t="n">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -3354,17 +3488,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>S-447/26-PL</t>
+          <t>CD-8/26-PL</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>MENDOZA Y OTROS: REPRODUCE PROYECTO DE LEY QUE DECLARA PATRIMONIO INMATERIAL CULTURAL Y NATURAL DE LA NACION, EN LOS TERMINOS DE LA LEY 26.118, AL "CHAKU", PRACTICA ANCESTRAL INCAICA DE CAPTURA, ESQUILA Y LIBERACIÓN DE VICUÑAS. (REF. S. 830/24).</t>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LAS LEYES 11683 Y 27799 (T.O. 1998 Y S/M) RELATIVAS A LA MODALIDAD SIMPLIFICADA DE DECLARACION JURADA DEL IMPUESTO A LAS GANANCIAS Y EN MATERIA DE PRESCRIPCION TRIBUTARIA, Y 25.191 REFERENTE AL REGIMEN SANCIONATORIO.</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3383,7 +3517,7 @@
         <v>2026</v>
       </c>
       <c r="B78" t="n">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -3392,17 +3526,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>CD-8/26-PL</t>
+          <t>S-336/25-PD</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LAS LEYES 11683 Y 27799 (T.O. 1998 Y S/M) RELATIVAS A LA MODALIDAD SIMPLIFICADA DE DECLARACION JURADA DEL IMPUESTO A LAS GANANCIAS Y EN MATERIA DE PRESCRIPCION TRIBUTARIA, Y 25.191 REFERENTE AL REGIMEN SANCIONATORIO.</t>
+          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL "PROYECTO INSTITUCIONAL DE CONVIVENCIA, UNA INVITACIÓN A INNOVAR- VALORES EN ACCIÓN-", PARA IMPLEMENTAR EN SUS NIVELES INICIAL, PRIMARIO Y SECUNDARIO, DISEÑADO POR EL COLEGIO "LA MERCED" DE LA CDAD. DE RIO CUARTO, PROV. DE CÓRDOBA.</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3421,7 +3555,7 @@
         <v>2026</v>
       </c>
       <c r="B79" t="n">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -3430,12 +3564,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>S-336/25-PD</t>
+          <t>S-837/25-PD</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL "PROYECTO INSTITUCIONAL DE CONVIVENCIA, UNA INVITACIÓN A INNOVAR- VALORES EN ACCIÓN-", PARA IMPLEMENTAR EN SUS NIVELES INICIAL, PRIMARIO Y SECUNDARIO, DISEÑADO POR EL COLEGIO "LA MERCED" DE LA CDAD. DE RIO CUARTO, PROV. DE CÓRDOBA.</t>
+          <t>ROJAS DECUT: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA DE EDUCACION FINANCIERA "CUENTAS SANAS" DE LA FUNDACION MACRO.</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3459,7 +3593,7 @@
         <v>2026</v>
       </c>
       <c r="B80" t="n">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -3468,17 +3602,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>S-837/25-PD</t>
+          <t>S-1469/25-PD</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ROJAS DECUT: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA DE EDUCACION FINANCIERA "CUENTAS SANAS" DE LA FUNDACION MACRO.</t>
+          <t>HUALA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCE A LA ESCRITORA OLGA LILIANA REINOSO POR SU TRAYECTORIA Y APORTE A LA CULTURA.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3497,7 +3631,7 @@
         <v>2026</v>
       </c>
       <c r="B81" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -3506,17 +3640,17 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>S-1469/25-PD</t>
+          <t>S-1577/25-PD</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>HUALA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCE A LA ESCRITORA OLGA LILIANA REINOSO POR SU TRAYECTORIA Y APORTE A LA CULTURA.</t>
+          <t>LEWANDOWSKI: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA TRAYECTORIA DEL MUSICO MIGUEL FIGUEROA Y SU CONJUNTO "AMANECER CAMPERO", CON LA DIFUSION DEL CHAMAME EN EL AMBITO NACIONAL E INTERNACIONAL.</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3535,7 +3669,7 @@
         <v>2026</v>
       </c>
       <c r="B82" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -3544,12 +3678,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>S-1577/25-PD</t>
+          <t>S-1601/25-PD</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>LEWANDOWSKI: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA TRAYECTORIA DEL MUSICO MIGUEL FIGUEROA Y SU CONJUNTO "AMANECER CAMPERO", CON LA DIFUSION DEL CHAMAME EN EL AMBITO NACIONAL E INTERNACIONAL.</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL EVENTO "CONVINART", RECONOCIENDO SU APORTE A LA DIFUSION DE LA CULTURA, EL ARTE Y LA IDENTIDAD NACIONAL.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3573,7 +3707,7 @@
         <v>2026</v>
       </c>
       <c r="B83" t="n">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -3582,12 +3716,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>S-1601/25-PD</t>
+          <t>S-1799/25-PD</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL EVENTO "CONVINART", RECONOCIENDO SU APORTE A LA DIFUSION DE LA CULTURA, EL ARTE Y LA IDENTIDAD NACIONAL.</t>
+          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE RECONOCE COMO VALOR HISTORICO Y CULTURAL AL MONOLITO DE LOMA BLANCA, EN LA LOCALIDAD DE OLTA, PROV. DE LA RIOJA.</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3611,7 +3745,7 @@
         <v>2026</v>
       </c>
       <c r="B84" t="n">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -3620,12 +3754,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>S-1799/25-PD</t>
+          <t>S-1987/25-PD</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE RECONOCE COMO VALOR HISTORICO Y CULTURAL AL MONOLITO DE LOMA BLANCA, EN LA LOCALIDAD DE OLTA, PROV. DE LA RIOJA.</t>
+          <t>GALARETTO: PROYECTO DE DECLARACION QUE DECLARA DE INTERES CULTURAL Y EDUCATIVO LA OBRA "DANZAS, BAILES Y COSTUMBRES DEL LITORAL ARGENTINO" DE LOS AUTORES CLAUDIA L. GARCIA Y ENRIQUE A. PIÑEYRO PUBLICADA POR EDITORIAL AUTORES ARGENTINOS EN 2025.</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3649,7 +3783,7 @@
         <v>2026</v>
       </c>
       <c r="B85" t="n">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -3658,12 +3792,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>S-1987/25-PD</t>
+          <t>S-709/26-PD</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>GALARETTO: PROYECTO DE DECLARACION QUE DECLARA DE INTERES CULTURAL Y EDUCATIVO LA OBRA "DANZAS, BAILES Y COSTUMBRES DEL LITORAL ARGENTINO" DE LOS AUTORES CLAUDIA L. GARCIA Y ENRIQUE A. PIÑEYRO PUBLICADA POR EDITORIAL AUTORES ARGENTINOS EN 2025.</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3687,7 +3821,7 @@
         <v>2026</v>
       </c>
       <c r="B86" t="n">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -3696,12 +3830,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>S-709/26-PD</t>
+          <t>S-735/26-PD</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
+          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3725,7 +3859,7 @@
         <v>2026</v>
       </c>
       <c r="B87" t="n">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -3734,12 +3868,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>S-735/26-PD</t>
+          <t>S-892/26-PD</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
+          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3763,7 +3897,7 @@
         <v>2026</v>
       </c>
       <c r="B88" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -3772,12 +3906,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>S-892/26-PD</t>
+          <t>S-900/26-PD</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
+          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3801,7 +3935,7 @@
         <v>2026</v>
       </c>
       <c r="B89" t="n">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -3810,12 +3944,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>S-900/26-PD</t>
+          <t>S-934/26-PD</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3839,7 +3973,7 @@
         <v>2026</v>
       </c>
       <c r="B90" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -3848,12 +3982,13 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>S-934/26-PD</t>
+          <t>S-2149/25-PD
+S-300/26-PD</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+          <t>CAPITANICH: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA BIENAL INTERNACIONAL DE ESCULTURAS DE CHACO 2026, A REALIZARSE EN LA CDAD. DE RESISTENCIA, DEL 11 AL 19 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3877,7 +4012,7 @@
         <v>2026</v>
       </c>
       <c r="B91" t="n">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -3886,13 +4021,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>S-2149/25-PD
-S-300/26-PD</t>
+          <t>S-935/26-PD</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>CAPITANICH: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA BIENAL INTERNACIONAL DE ESCULTURAS DE CHACO 2026, A REALIZARSE EN LA CDAD. DE RESISTENCIA, DEL 11 AL 19 DE JULIO DE 2026.</t>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3916,7 +4050,7 @@
         <v>2026</v>
       </c>
       <c r="B92" t="n">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -3925,12 +4059,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>S-935/26-PD</t>
+          <t>S-1006/26-PD</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
+          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3954,7 +4088,7 @@
         <v>2026</v>
       </c>
       <c r="B93" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -3963,12 +4097,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>S-1006/26-PD</t>
+          <t>S-1017/26-PD</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
+          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3992,7 +4126,7 @@
         <v>2026</v>
       </c>
       <c r="B94" t="n">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -4001,12 +4135,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>S-1017/26-PD</t>
+          <t>S-1020/26-PD</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4030,7 +4164,7 @@
         <v>2026</v>
       </c>
       <c r="B95" t="n">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -4039,12 +4173,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>S-1020/26-PD</t>
+          <t>S-1037/26-PD</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4068,7 +4202,7 @@
         <v>2026</v>
       </c>
       <c r="B96" t="n">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -4077,12 +4211,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>S-1037/26-PD</t>
+          <t>S-1038/26-PD</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
+          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4106,7 +4240,7 @@
         <v>2026</v>
       </c>
       <c r="B97" t="n">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -4115,12 +4249,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>S-1038/26-PD</t>
+          <t>S-1104/26-PD</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
+          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4144,7 +4278,7 @@
         <v>2026</v>
       </c>
       <c r="B98" t="n">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -4153,12 +4287,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>S-1104/26-PD</t>
+          <t>S-1122/26-PD</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
+          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4182,7 +4316,7 @@
         <v>2026</v>
       </c>
       <c r="B99" t="n">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -4191,12 +4325,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>S-1122/26-PD</t>
+          <t>S-1029/26-PD</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4220,7 +4354,7 @@
         <v>2026</v>
       </c>
       <c r="B100" t="n">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -4229,12 +4363,13 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>S-1029/26-PD</t>
+          <t>S-1154/26-PD
+S-1166/26-PD</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+          <t>ATAUCHE: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES EL NUEVO ANIVERSARIO DEL EXODO JUJEÑO, EL 23 DE AGOSTO DE 2026.</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4258,7 +4393,7 @@
         <v>2026</v>
       </c>
       <c r="B101" t="n">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -4267,13 +4402,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>S-1154/26-PD
-S-1166/26-PD</t>
+          <t>S-1165/26-PD</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>ATAUCHE: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES EL NUEVO ANIVERSARIO DEL EXODO JUJEÑO, EL 23 DE AGOSTO DE 2026.</t>
+          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4293,30 +4427,39 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B102" t="n">
-        <v>397</v>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>ANEXO</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>S-1165/26-PD</t>
+          <t>PE-150/19-PL</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
+          <t>MENSAJE N° 111/19 Y PROYECTO DE LEY QUE APRUEBA LA REFORMA DEL CONVENIO INTERAMERICANO SOBRE PERMISO INTERNACIONAL DE RADIOAFICIONADO, ADOPTADO EN LA CDAD. DE WASHINGTON D.C., ESTADOS UNIDOS DE AMERICA, EL 4 DE JUNIO DE 2018.</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE RELACIONES EXTERIORES Y CULTO -</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4325,6 +4468,100 @@
         </is>
       </c>
       <c r="I102" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>PE-145/24-AC</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>MENSAJE Nº 69/24 QUE SOLICITA ACUERDO PARA PROMOVER AL GRADO INMEDIATO SUPERIOR, CON FECHA 31 DE DICIEMBRE DE 2024, A PERSONAL MILITAR SUPERIOR DE LA FUERZA AÈREA ARGENTINA.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS - DE ACUERDOS -</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>27/03/2026</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>PE-96/22-AC</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 75/22 QUE SOLICITA ACUERDO PARA PROMOVER AL GRADO INMEDIATO SUPERIOR AL PERSONAL MILITAR SUPERIOR DE LA FUERZA AÉREA ARGENTINA, CON FECHA 31 DE DICIEMBRE DE 2021</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS - DE ACUERDOS - DE ACUERDOS -</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>27/03/2026</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4378,162 +4615,198 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A103" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId238"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(ayuda-memoria): agrega el dictamen de mayoría de la OD 113/26
Sólo había cargado el anexo (minoría); con el de mayoría (PE-150/19-PL,
mismo expediente) ahora se fusionan en una sola tarjeta como corresponde
-- mayoría con sus firmantes, minoría anidada con los suyos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4562,6 +4562,49 @@
         </is>
       </c>
       <c r="I104" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B105" t="n">
+        <v>113</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>PE-150/19-PL</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 111/19 Y PROYECTO DE LEY QUE APRUEBA LA REFORMA DEL CONVENIO INTERAMERICANO SOBRE PERMISO INTERNACIONAL DE RADIOAFICIONADO, ADOPTADO EN LA CDAD. DE WASHINGTON D.C., ESTADOS UNIDOS DE AMERICA, EL 4 DE JUNIO DE 2018.</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>DE RELACIONES EXTERIORES Y CULTO -</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4807,6 +4850,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="rId236"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId237"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId240"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 05:42 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>ANEXO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3421,7 +3421,7 @@
         <v>2026</v>
       </c>
       <c r="B79" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -3430,17 +3430,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>S-336/25-PD</t>
+          <t>CD-8/26-PL</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL "PROYECTO INSTITUCIONAL DE CONVIVENCIA, UNA INVITACIÓN A INNOVAR- VALORES EN ACCIÓN-", PARA IMPLEMENTAR EN SUS NIVELES INICIAL, PRIMARIO Y SECUNDARIO, DISEÑADO POR EL COLEGIO "LA MERCED" DE LA CDAD. DE RIO CUARTO, PROV. DE CÓRDOBA.</t>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LAS LEYES 11683 Y 27799 (T.O. 1998 Y S/M) RELATIVAS A LA MODALIDAD SIMPLIFICADA DE DECLARACION JURADA DEL IMPUESTO A LAS GANANCIAS Y EN MATERIA DE PRESCRIPCION TRIBUTARIA, Y 25.191 REFERENTE AL REGIMEN SANCIONATORIO.</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3459,7 +3459,7 @@
         <v>2026</v>
       </c>
       <c r="B80" t="n">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -3468,12 +3468,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>S-837/25-PD</t>
+          <t>S-336/25-PD</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ROJAS DECUT: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA DE EDUCACION FINANCIERA "CUENTAS SANAS" DE LA FUNDACION MACRO.</t>
+          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL "PROYECTO INSTITUCIONAL DE CONVIVENCIA, UNA INVITACIÓN A INNOVAR- VALORES EN ACCIÓN-", PARA IMPLEMENTAR EN SUS NIVELES INICIAL, PRIMARIO Y SECUNDARIO, DISEÑADO POR EL COLEGIO "LA MERCED" DE LA CDAD. DE RIO CUARTO, PROV. DE CÓRDOBA.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3497,7 +3497,7 @@
         <v>2026</v>
       </c>
       <c r="B81" t="n">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -3506,17 +3506,17 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>S-1469/25-PD</t>
+          <t>S-837/25-PD</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>HUALA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCE A LA ESCRITORA OLGA LILIANA REINOSO POR SU TRAYECTORIA Y APORTE A LA CULTURA.</t>
+          <t>ROJAS DECUT: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA DE EDUCACION FINANCIERA "CUENTAS SANAS" DE LA FUNDACION MACRO.</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3535,7 +3535,7 @@
         <v>2026</v>
       </c>
       <c r="B82" t="n">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -3544,17 +3544,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>S-1577/25-PD</t>
+          <t>S-1469/25-PD</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>LEWANDOWSKI: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA TRAYECTORIA DEL MUSICO MIGUEL FIGUEROA Y SU CONJUNTO "AMANECER CAMPERO", CON LA DIFUSION DEL CHAMAME EN EL AMBITO NACIONAL E INTERNACIONAL.</t>
+          <t>HUALA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCE A LA ESCRITORA OLGA LILIANA REINOSO POR SU TRAYECTORIA Y APORTE A LA CULTURA.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3573,7 +3573,7 @@
         <v>2026</v>
       </c>
       <c r="B83" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -3582,12 +3582,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>S-1601/25-PD</t>
+          <t>S-1577/25-PD</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL EVENTO "CONVINART", RECONOCIENDO SU APORTE A LA DIFUSION DE LA CULTURA, EL ARTE Y LA IDENTIDAD NACIONAL.</t>
+          <t>LEWANDOWSKI: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA TRAYECTORIA DEL MUSICO MIGUEL FIGUEROA Y SU CONJUNTO "AMANECER CAMPERO", CON LA DIFUSION DEL CHAMAME EN EL AMBITO NACIONAL E INTERNACIONAL.</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3611,7 +3611,7 @@
         <v>2026</v>
       </c>
       <c r="B84" t="n">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -3620,12 +3620,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>S-1799/25-PD</t>
+          <t>S-1601/25-PD</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE RECONOCE COMO VALOR HISTORICO Y CULTURAL AL MONOLITO DE LOMA BLANCA, EN LA LOCALIDAD DE OLTA, PROV. DE LA RIOJA.</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL EVENTO "CONVINART", RECONOCIENDO SU APORTE A LA DIFUSION DE LA CULTURA, EL ARTE Y LA IDENTIDAD NACIONAL.</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3649,7 +3649,7 @@
         <v>2026</v>
       </c>
       <c r="B85" t="n">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -3658,12 +3658,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>S-1987/25-PD</t>
+          <t>S-1799/25-PD</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>GALARETTO: PROYECTO DE DECLARACION QUE DECLARA DE INTERES CULTURAL Y EDUCATIVO LA OBRA "DANZAS, BAILES Y COSTUMBRES DEL LITORAL ARGENTINO" DE LOS AUTORES CLAUDIA L. GARCIA Y ENRIQUE A. PIÑEYRO PUBLICADA POR EDITORIAL AUTORES ARGENTINOS EN 2025.</t>
+          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE RECONOCE COMO VALOR HISTORICO Y CULTURAL AL MONOLITO DE LOMA BLANCA, EN LA LOCALIDAD DE OLTA, PROV. DE LA RIOJA.</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3687,7 +3687,7 @@
         <v>2026</v>
       </c>
       <c r="B86" t="n">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -3696,12 +3696,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>S-709/26-PD</t>
+          <t>S-1987/25-PD</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
+          <t>GALARETTO: PROYECTO DE DECLARACION QUE DECLARA DE INTERES CULTURAL Y EDUCATIVO LA OBRA "DANZAS, BAILES Y COSTUMBRES DEL LITORAL ARGENTINO" DE LOS AUTORES CLAUDIA L. GARCIA Y ENRIQUE A. PIÑEYRO PUBLICADA POR EDITORIAL AUTORES ARGENTINOS EN 2025.</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3725,7 +3725,7 @@
         <v>2026</v>
       </c>
       <c r="B87" t="n">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -3734,12 +3734,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>S-735/26-PD</t>
+          <t>S-709/26-PD</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3763,7 +3763,7 @@
         <v>2026</v>
       </c>
       <c r="B88" t="n">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -3772,12 +3772,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>S-892/26-PD</t>
+          <t>S-735/26-PD</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
+          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3801,7 +3801,7 @@
         <v>2026</v>
       </c>
       <c r="B89" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -3810,12 +3810,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>S-900/26-PD</t>
+          <t>S-892/26-PD</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
+          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3839,7 +3839,7 @@
         <v>2026</v>
       </c>
       <c r="B90" t="n">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -3848,12 +3848,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>S-934/26-PD</t>
+          <t>S-900/26-PD</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3877,60 +3877,60 @@
         <v>2026</v>
       </c>
       <c r="B91" t="n">
+        <v>385</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>S-934/26-PD</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B92" t="n">
         <v>386</v>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
         <is>
           <t>S-2149/25-PD
 S-300/26-PD</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>CAPITANICH: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA BIENAL INTERNACIONAL DE ESCULTURAS DE CHACO 2026, A REALIZARSE EN LA CDAD. DE RESISTENCIA, DEL 11 AL 19 DE JULIO DE 2026.</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B92" t="n">
-        <v>387</v>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>S-935/26-PD</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3954,7 +3954,7 @@
         <v>2026</v>
       </c>
       <c r="B93" t="n">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -3963,12 +3963,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>S-1006/26-PD</t>
+          <t>S-935/26-PD</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3992,7 +3992,7 @@
         <v>2026</v>
       </c>
       <c r="B94" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -4001,12 +4001,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>S-1017/26-PD</t>
+          <t>S-1006/26-PD</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4030,7 +4030,7 @@
         <v>2026</v>
       </c>
       <c r="B95" t="n">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -4039,12 +4039,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>S-1020/26-PD</t>
+          <t>S-1017/26-PD</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
+          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4068,7 +4068,7 @@
         <v>2026</v>
       </c>
       <c r="B96" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -4077,12 +4077,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>S-1037/26-PD</t>
+          <t>S-1020/26-PD</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
+          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4106,7 +4106,7 @@
         <v>2026</v>
       </c>
       <c r="B97" t="n">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -4115,12 +4115,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>S-1038/26-PD</t>
+          <t>S-1037/26-PD</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4144,7 +4144,7 @@
         <v>2026</v>
       </c>
       <c r="B98" t="n">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -4153,12 +4153,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>S-1104/26-PD</t>
+          <t>S-1038/26-PD</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
+          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4182,7 +4182,7 @@
         <v>2026</v>
       </c>
       <c r="B99" t="n">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -4191,12 +4191,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>S-1122/26-PD</t>
+          <t>S-1104/26-PD</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4220,7 +4220,7 @@
         <v>2026</v>
       </c>
       <c r="B100" t="n">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>S-1029/26-PD</t>
+          <t>S-1122/26-PD</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4258,60 +4258,60 @@
         <v>2026</v>
       </c>
       <c r="B101" t="n">
+        <v>395</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>S-1029/26-PD</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B102" t="n">
         <v>396</v>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
         <is>
           <t>S-1154/26-PD
 S-1166/26-PD</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>ATAUCHE: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES EL NUEVO ANIVERSARIO DEL EXODO JUJEÑO, EL 23 DE AGOSTO DE 2026.</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B102" t="n">
-        <v>397</v>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>S-1165/26-PD</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4335,7 +4335,7 @@
         <v>2026</v>
       </c>
       <c r="B103" t="n">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -4344,17 +4344,17 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>S-1152/25-PD</t>
+          <t>S-1165/26-PD</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>ATAUCHE: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA RADIAL "VIAJANDO POR ARGENTINA".</t>
+          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4373,7 +4373,7 @@
         <v>2026</v>
       </c>
       <c r="B104" t="n">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -4382,12 +4382,12 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>S-1563/25-PD</t>
+          <t>S-1152/25-PD</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LOS PREMIOS PRISMA 2025, A REALIZARSE EN LA CDAD. DE POSADAS, PROV. DE MISIONES, EL 18 DE OCTUBRE.</t>
+          <t>ATAUCHE: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA RADIAL "VIAJANDO POR ARGENTINA".</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -4411,7 +4411,7 @@
         <v>2026</v>
       </c>
       <c r="B105" t="n">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -4420,12 +4420,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>S-1647/25-PD</t>
+          <t>S-1563/25-PD</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>LEAVY: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA "SALTA ES UNA CANCION" QUE SE EMITE POR LA TELEVISION SALTEÑA DESDE 1997.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LOS PREMIOS PRISMA 2025, A REALIZARSE EN LA CDAD. DE POSADAS, PROV. DE MISIONES, EL 18 DE OCTUBRE.</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4449,74 +4449,151 @@
         <v>2026</v>
       </c>
       <c r="B106" t="n">
+        <v>400</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>S-1647/25-PD</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LEAVY: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA "SALTA ES UNA CANCION" QUE SE EMITE POR LA TELEVISION SALTEÑA DESDE 1997.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B107" t="n">
         <v>401</v>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
         <is>
           <t>S-931/25-PD
 S-998/26-PD</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="E107" t="inlineStr">
         <is>
           <t>VISCHI: PROYECTO DE DECLARACIÓN QUE ADHIERE A LA CELEBRACIÓN DEL DIA DEL PERIODISTA, EL 7 DE JUNIO.</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
+      <c r="F107" t="inlineStr">
         <is>
           <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B107" t="n">
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B108" t="n">
         <v>402</v>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ANEXO</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
         <is>
           <t>CD-3/26-PL
 S-909/26-PL</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E108" t="inlineStr">
         <is>
           <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA LEY 25.565, DE PRESUPUESTO GENERAL DE GASTOS DE LA ADM. NACIONAL PARA EL EJERCICIO 2002 SOBRE READECUACION DEL REGIMEN DE SUBSIDIOS A LOS CONSUMOS RESIDENCIALES DE GAS NATURAL EN ZONAS FRIAS, REGULARIZACION DE DEUDAS ELECTRICAS Y DEROGA LOS DECRETOS 277/2022 Y 929/2013.</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
+      <c r="F108" t="inlineStr">
         <is>
           <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B109" t="n">
+        <v>402</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>CD-3/26-PL
+S-909/26-PL</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA LEY 25.565, DE PRESUPUESTO GENERAL DE GASTOS DE LA ADM. NACIONAL PARA EL EJERCICIO 2002 SOBRE READECUACION DEL REGIMEN DE SUBSIDIOS A LOS CONSUMOS RESIDENCIALES DE GAS NATURAL EN ZONAS FRIAS, REGULARIZACION DE DEUDAS ELECTRICAS Y DEROGA LOS DECRETOS 277/2022 Y 929/2013.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES - DE PRESUPUESTO Y HACIENDA -</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4736,6 +4813,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId210"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId211"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId216"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática 2026-09-23 05:39 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4594,6 +4594,120 @@
         </is>
       </c>
       <c r="I109" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B110" t="n">
+        <v>403</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>S-229/25-PC</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA UNA CAMPAÑA MASIVA DE COMUNICACIÓN A TRAVÉS DE LOS MEDIOS DE COMUNICACIÓN Y EN LAS ESCUELAS PÚBLICAS Y PRIVADAS ORIENTADA A LA PREVENCIÓN Y CONCIENTIZACIÓN SOBRE EL "PHISHING".</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B111" t="n">
+        <v>404</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>S-1254/25-PC</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA SE REALICE UNA CAMPAÑA EN MEDIOS DE COMUNICACIÓN Y ESTABLECIMIENTOS EDUCATIVOS PÚBLICOS Y PRIVADOS DE PREVENCIÓN Y CONCIENTIZACIÓN SOBRE LA VIOLENCIA EN ENTORNOS DIGITALES.</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B112" t="n">
+        <v>405</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>S-68/26-PC</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA LA REALIZACION DE UNA CAMPAÑA DE COMUNICACIÓN ORIENTADA A LA PREVENCION Y CONCIENTIZACION DE LA LUDOPATIA INFANTIL, Y DE LA AUTODEPENDENCIA A DISPOSITIVOS MOVILES, VIDEOJUEGOS Y REDES SOCIALES EN MENORES DE 18 AÑOS.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4817,6 +4931,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId214"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId215"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I110" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId222"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 06:03 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:I114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4708,6 +4708,82 @@
         </is>
       </c>
       <c r="I112" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B113" t="n">
+        <v>406</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>S-881/26-PD</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL QUINCUAGESIMO QUINTO ANIVERSARIO DEL PROGRAMA "FORMULA TUERCA Y TODOS LOS DEPORTES", EMITIDO POR LT4 RADIODIFUSORA MISIONES, PROV. HOMONIMA, EL 1° DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B114" t="n">
+        <v>407</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>PE-133/26-AC</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 138/26 QUE SOLICITA ACUERDO PARA PROMOVER AL GRADO INMEDIATO SUPERIOR, AL 31 DE DICIEMBRE DE 2025, AL GENERAL DE BRIGADA SEBASTIAN IGNACIO IBAÑEZ.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS -</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -4937,6 +5013,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId220"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId221"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I113" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId226"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática 2026-09-25 06:00 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I114"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>ANEXO</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3231,7 +3231,7 @@
         <v>2026</v>
       </c>
       <c r="B74" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -3240,17 +3240,17 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>S-1643/25-PL</t>
+          <t>CD-7/26-PL</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>VISCHI: REPRODUCE PROYECTO DE LEY QUE DECLARA BIEN HISTORICO NACIONAL, EN LOS TERMINOS DE LA LEY 12.665 Y S/M., AL INMUEBLE IDENTIFICADO COMO EX "HOTEL DE INMIGRANTES- EX OFICINAS DE PUENTES Y CAMINOS DE GOYA", SITO EN LA MANZANA N° 497, ENTRE LAS CALLES CAÁ GUAZU Y AV. SARMIENTO DE LA CIUDAD DE GOYA, PROV. DE CORRIENTES. (REF. S.1422/22)</t>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA CARTA ORGANICA DEL BANCO CENTRAL DE LA REPUBLICA ARGENTINA.</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE ECONOMÍA NACIONAL E INVERSIÓN - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3269,7 +3269,7 @@
         <v>2026</v>
       </c>
       <c r="B75" t="n">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -3278,12 +3278,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>S-124/26-PL</t>
+          <t>S-1643/25-PL</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE DECLARA MONUMENTO HISTORICO NACIONAL AL CEMENTERIO OESTE DE SAN MIGUEL DE TUCUMAN, PROV. DE TUCUMAN.</t>
+          <t>VISCHI: REPRODUCE PROYECTO DE LEY QUE DECLARA BIEN HISTORICO NACIONAL, EN LOS TERMINOS DE LA LEY 12.665 Y S/M., AL INMUEBLE IDENTIFICADO COMO EX "HOTEL DE INMIGRANTES- EX OFICINAS DE PUENTES Y CAMINOS DE GOYA", SITO EN LA MANZANA N° 497, ENTRE LAS CALLES CAÁ GUAZU Y AV. SARMIENTO DE LA CIUDAD DE GOYA, PROV. DE CORRIENTES. (REF. S.1422/22)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3307,7 +3307,7 @@
         <v>2026</v>
       </c>
       <c r="B76" t="n">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -3316,12 +3316,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>S-255/26-PL</t>
+          <t>S-124/26-PL</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>FAMA: REPRODUCE PROYECTO DE LEY QUE MODIFICA SU SIMILAR 26.206 -EDUCACION NACIONAL-  RESPECTO DE PROMOVER EL DESARROLLO DE LA EDUCACION EMOCIONAL. (REF. S. 752/22)</t>
+          <t>AVILA: PROYECTO DE LEY QUE DECLARA MONUMENTO HISTORICO NACIONAL AL CEMENTERIO OESTE DE SAN MIGUEL DE TUCUMAN, PROV. DE TUCUMAN.</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3345,7 +3345,7 @@
         <v>2026</v>
       </c>
       <c r="B77" t="n">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -3354,12 +3354,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>S-447/26-PL</t>
+          <t>S-255/26-PL</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>MENDOZA Y OTROS: REPRODUCE PROYECTO DE LEY QUE DECLARA PATRIMONIO INMATERIAL CULTURAL Y NATURAL DE LA NACION, EN LOS TERMINOS DE LA LEY 26.118, AL "CHAKU", PRACTICA ANCESTRAL INCAICA DE CAPTURA, ESQUILA Y LIBERACIÓN DE VICUÑAS. (REF. S. 830/24).</t>
+          <t>FAMA: REPRODUCE PROYECTO DE LEY QUE MODIFICA SU SIMILAR 26.206 -EDUCACION NACIONAL-  RESPECTO DE PROMOVER EL DESARROLLO DE LA EDUCACION EMOCIONAL. (REF. S. 752/22)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3383,26 +3383,26 @@
         <v>2026</v>
       </c>
       <c r="B78" t="n">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ANEXO</t>
+          <t>NORMAL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>CD-8/26-PL</t>
+          <t>S-447/26-PL</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LAS LEYES 11683 Y 27799 (T.O. 1998 Y S/M) RELATIVAS A LA MODALIDAD SIMPLIFICADA DE DECLARACION JURADA DEL IMPUESTO A LAS GANANCIAS Y EN MATERIA DE PRESCRIPCION TRIBUTARIA, Y 25.191 REFERENTE AL REGIMEN SANCIONATORIO.</t>
+          <t>MENDOZA Y OTROS: REPRODUCE PROYECTO DE LEY QUE DECLARA PATRIMONIO INMATERIAL CULTURAL Y NATURAL DE LA NACION, EN LOS TERMINOS DE LA LEY 26.118, AL "CHAKU", PRACTICA ANCESTRAL INCAICA DE CAPTURA, ESQUILA Y LIBERACIÓN DE VICUÑAS. (REF. S. 830/24).</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>ANEXO</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3459,7 +3459,7 @@
         <v>2026</v>
       </c>
       <c r="B80" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -3468,17 +3468,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>S-336/25-PD</t>
+          <t>CD-8/26-PL</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL "PROYECTO INSTITUCIONAL DE CONVIVENCIA, UNA INVITACIÓN A INNOVAR- VALORES EN ACCIÓN-", PARA IMPLEMENTAR EN SUS NIVELES INICIAL, PRIMARIO Y SECUNDARIO, DISEÑADO POR EL COLEGIO "LA MERCED" DE LA CDAD. DE RIO CUARTO, PROV. DE CÓRDOBA.</t>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LAS LEYES 11683 Y 27799 (T.O. 1998 Y S/M) RELATIVAS A LA MODALIDAD SIMPLIFICADA DE DECLARACION JURADA DEL IMPUESTO A LAS GANANCIAS Y EN MATERIA DE PRESCRIPCION TRIBUTARIA, Y 25.191 REFERENTE AL REGIMEN SANCIONATORIO.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3497,7 +3497,7 @@
         <v>2026</v>
       </c>
       <c r="B81" t="n">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -3506,12 +3506,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>S-837/25-PD</t>
+          <t>S-336/25-PD</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ROJAS DECUT: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA DE EDUCACION FINANCIERA "CUENTAS SANAS" DE LA FUNDACION MACRO.</t>
+          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL "PROYECTO INSTITUCIONAL DE CONVIVENCIA, UNA INVITACIÓN A INNOVAR- VALORES EN ACCIÓN-", PARA IMPLEMENTAR EN SUS NIVELES INICIAL, PRIMARIO Y SECUNDARIO, DISEÑADO POR EL COLEGIO "LA MERCED" DE LA CDAD. DE RIO CUARTO, PROV. DE CÓRDOBA.</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3535,7 +3535,7 @@
         <v>2026</v>
       </c>
       <c r="B82" t="n">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -3544,17 +3544,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>S-1469/25-PD</t>
+          <t>S-837/25-PD</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>HUALA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCE A LA ESCRITORA OLGA LILIANA REINOSO POR SU TRAYECTORIA Y APORTE A LA CULTURA.</t>
+          <t>ROJAS DECUT: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA DE EDUCACION FINANCIERA "CUENTAS SANAS" DE LA FUNDACION MACRO.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3573,7 +3573,7 @@
         <v>2026</v>
       </c>
       <c r="B83" t="n">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -3582,17 +3582,17 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>S-1577/25-PD</t>
+          <t>S-1469/25-PD</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>LEWANDOWSKI: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA TRAYECTORIA DEL MUSICO MIGUEL FIGUEROA Y SU CONJUNTO "AMANECER CAMPERO", CON LA DIFUSION DEL CHAMAME EN EL AMBITO NACIONAL E INTERNACIONAL.</t>
+          <t>HUALA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCE A LA ESCRITORA OLGA LILIANA REINOSO POR SU TRAYECTORIA Y APORTE A LA CULTURA.</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3611,7 +3611,7 @@
         <v>2026</v>
       </c>
       <c r="B84" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -3620,12 +3620,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>S-1601/25-PD</t>
+          <t>S-1577/25-PD</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL EVENTO "CONVINART", RECONOCIENDO SU APORTE A LA DIFUSION DE LA CULTURA, EL ARTE Y LA IDENTIDAD NACIONAL.</t>
+          <t>LEWANDOWSKI: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA TRAYECTORIA DEL MUSICO MIGUEL FIGUEROA Y SU CONJUNTO "AMANECER CAMPERO", CON LA DIFUSION DEL CHAMAME EN EL AMBITO NACIONAL E INTERNACIONAL.</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3649,7 +3649,7 @@
         <v>2026</v>
       </c>
       <c r="B85" t="n">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -3658,12 +3658,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>S-1799/25-PD</t>
+          <t>S-1601/25-PD</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE RECONOCE COMO VALOR HISTORICO Y CULTURAL AL MONOLITO DE LOMA BLANCA, EN LA LOCALIDAD DE OLTA, PROV. DE LA RIOJA.</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL EVENTO "CONVINART", RECONOCIENDO SU APORTE A LA DIFUSION DE LA CULTURA, EL ARTE Y LA IDENTIDAD NACIONAL.</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3687,7 +3687,7 @@
         <v>2026</v>
       </c>
       <c r="B86" t="n">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -3696,12 +3696,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>S-1987/25-PD</t>
+          <t>S-1799/25-PD</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>GALARETTO: PROYECTO DE DECLARACION QUE DECLARA DE INTERES CULTURAL Y EDUCATIVO LA OBRA "DANZAS, BAILES Y COSTUMBRES DEL LITORAL ARGENTINO" DE LOS AUTORES CLAUDIA L. GARCIA Y ENRIQUE A. PIÑEYRO PUBLICADA POR EDITORIAL AUTORES ARGENTINOS EN 2025.</t>
+          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE RECONOCE COMO VALOR HISTORICO Y CULTURAL AL MONOLITO DE LOMA BLANCA, EN LA LOCALIDAD DE OLTA, PROV. DE LA RIOJA.</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3725,7 +3725,7 @@
         <v>2026</v>
       </c>
       <c r="B87" t="n">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -3734,12 +3734,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>S-709/26-PD</t>
+          <t>S-1987/25-PD</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
+          <t>GALARETTO: PROYECTO DE DECLARACION QUE DECLARA DE INTERES CULTURAL Y EDUCATIVO LA OBRA "DANZAS, BAILES Y COSTUMBRES DEL LITORAL ARGENTINO" DE LOS AUTORES CLAUDIA L. GARCIA Y ENRIQUE A. PIÑEYRO PUBLICADA POR EDITORIAL AUTORES ARGENTINOS EN 2025.</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3763,7 +3763,7 @@
         <v>2026</v>
       </c>
       <c r="B88" t="n">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -3772,12 +3772,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>S-735/26-PD</t>
+          <t>S-709/26-PD</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3801,7 +3801,7 @@
         <v>2026</v>
       </c>
       <c r="B89" t="n">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -3810,12 +3810,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>S-892/26-PD</t>
+          <t>S-735/26-PD</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
+          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3839,7 +3839,7 @@
         <v>2026</v>
       </c>
       <c r="B90" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -3848,12 +3848,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>S-900/26-PD</t>
+          <t>S-892/26-PD</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
+          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3877,7 +3877,7 @@
         <v>2026</v>
       </c>
       <c r="B91" t="n">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -3886,12 +3886,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>S-934/26-PD</t>
+          <t>S-900/26-PD</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3915,60 +3915,60 @@
         <v>2026</v>
       </c>
       <c r="B92" t="n">
+        <v>385</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>S-934/26-PD</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B93" t="n">
         <v>386</v>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
         <is>
           <t>S-2149/25-PD
 S-300/26-PD</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>CAPITANICH: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA BIENAL INTERNACIONAL DE ESCULTURAS DE CHACO 2026, A REALIZARSE EN LA CDAD. DE RESISTENCIA, DEL 11 AL 19 DE JULIO DE 2026.</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B93" t="n">
-        <v>387</v>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>S-935/26-PD</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3992,7 +3992,7 @@
         <v>2026</v>
       </c>
       <c r="B94" t="n">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -4001,12 +4001,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>S-1006/26-PD</t>
+          <t>S-935/26-PD</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4030,7 +4030,7 @@
         <v>2026</v>
       </c>
       <c r="B95" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -4039,12 +4039,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>S-1017/26-PD</t>
+          <t>S-1006/26-PD</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4068,7 +4068,7 @@
         <v>2026</v>
       </c>
       <c r="B96" t="n">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -4077,12 +4077,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>S-1020/26-PD</t>
+          <t>S-1017/26-PD</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
+          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4106,7 +4106,7 @@
         <v>2026</v>
       </c>
       <c r="B97" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -4115,12 +4115,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>S-1037/26-PD</t>
+          <t>S-1020/26-PD</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
+          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4144,7 +4144,7 @@
         <v>2026</v>
       </c>
       <c r="B98" t="n">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -4153,12 +4153,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>S-1038/26-PD</t>
+          <t>S-1037/26-PD</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4182,7 +4182,7 @@
         <v>2026</v>
       </c>
       <c r="B99" t="n">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -4191,12 +4191,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>S-1104/26-PD</t>
+          <t>S-1038/26-PD</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
+          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4220,7 +4220,7 @@
         <v>2026</v>
       </c>
       <c r="B100" t="n">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>S-1122/26-PD</t>
+          <t>S-1104/26-PD</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4258,7 +4258,7 @@
         <v>2026</v>
       </c>
       <c r="B101" t="n">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -4267,12 +4267,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>S-1029/26-PD</t>
+          <t>S-1122/26-PD</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4296,60 +4296,60 @@
         <v>2026</v>
       </c>
       <c r="B102" t="n">
+        <v>395</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>S-1029/26-PD</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B103" t="n">
         <v>396</v>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
         <is>
           <t>S-1154/26-PD
 S-1166/26-PD</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>ATAUCHE: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES EL NUEVO ANIVERSARIO DEL EXODO JUJEÑO, EL 23 DE AGOSTO DE 2026.</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B103" t="n">
-        <v>397</v>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>S-1165/26-PD</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4373,7 +4373,7 @@
         <v>2026</v>
       </c>
       <c r="B104" t="n">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -4382,17 +4382,17 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>S-1152/25-PD</t>
+          <t>S-1165/26-PD</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>ATAUCHE: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA RADIAL "VIAJANDO POR ARGENTINA".</t>
+          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4411,7 +4411,7 @@
         <v>2026</v>
       </c>
       <c r="B105" t="n">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -4420,12 +4420,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>S-1563/25-PD</t>
+          <t>S-1152/25-PD</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LOS PREMIOS PRISMA 2025, A REALIZARSE EN LA CDAD. DE POSADAS, PROV. DE MISIONES, EL 18 DE OCTUBRE.</t>
+          <t>ATAUCHE: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA RADIAL "VIAJANDO POR ARGENTINA".</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4449,7 +4449,7 @@
         <v>2026</v>
       </c>
       <c r="B106" t="n">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -4458,12 +4458,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>S-1647/25-PD</t>
+          <t>S-1563/25-PD</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>LEAVY: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA "SALTA ES UNA CANCION" QUE SE EMITE POR LA TELEVISION SALTEÑA DESDE 1997.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LOS PREMIOS PRISMA 2025, A REALIZARSE EN LA CDAD. DE POSADAS, PROV. DE MISIONES, EL 18 DE OCTUBRE.</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4487,143 +4487,143 @@
         <v>2026</v>
       </c>
       <c r="B107" t="n">
+        <v>400</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>S-1647/25-PD</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LEAVY: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA "SALTA ES UNA CANCION" QUE SE EMITE POR LA TELEVISION SALTEÑA DESDE 1997.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B108" t="n">
         <v>401</v>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
         <is>
           <t>S-931/25-PD
 S-998/26-PD</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E108" t="inlineStr">
         <is>
           <t>VISCHI: PROYECTO DE DECLARACIÓN QUE ADHIERE A LA CELEBRACIÓN DEL DIA DEL PERIODISTA, EL 7 DE JUNIO.</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
+      <c r="F108" t="inlineStr">
         <is>
           <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B108" t="n">
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B109" t="n">
         <v>402</v>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>ANEXO</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D109" t="inlineStr">
         <is>
           <t>CD-3/26-PL
 S-909/26-PL</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA LEY 25.565, DE PRESUPUESTO GENERAL DE GASTOS DE LA ADM. NACIONAL PARA EL EJERCICIO 2002 SOBRE READECUACION DEL REGIMEN DE SUBSIDIOS A LOS CONSUMOS RESIDENCIALES DE GAS NATURAL EN ZONAS FRIAS, REGULARIZACION DE DEUDAS ELECTRICAS Y DEROGA LOS DECRETOS 277/2022 Y 929/2013.</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B109" t="n">
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B110" t="n">
         <v>402</v>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
         <is>
           <t>CD-3/26-PL
 S-909/26-PL</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E110" t="inlineStr">
         <is>
           <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA LEY 25.565, DE PRESUPUESTO GENERAL DE GASTOS DE LA ADM. NACIONAL PARA EL EJERCICIO 2002 SOBRE READECUACION DEL REGIMEN DE SUBSIDIOS A LOS CONSUMOS RESIDENCIALES DE GAS NATURAL EN ZONAS FRIAS, REGULARIZACION DE DEUDAS ELECTRICAS Y DEROGA LOS DECRETOS 277/2022 Y 929/2013.</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
+      <c r="F110" t="inlineStr">
         <is>
           <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES - DE PRESUPUESTO Y HACIENDA -</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B110" t="n">
-        <v>403</v>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>S-229/25-PC</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA UNA CAMPAÑA MASIVA DE COMUNICACIÓN A TRAVÉS DE LOS MEDIOS DE COMUNICACIÓN Y EN LAS ESCUELAS PÚBLICAS Y PRIVADAS ORIENTADA A LA PREVENCIÓN Y CONCIENTIZACIÓN SOBRE EL "PHISHING".</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -4642,7 +4642,7 @@
         <v>2026</v>
       </c>
       <c r="B111" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -4651,12 +4651,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>S-1254/25-PC</t>
+          <t>S-229/25-PC</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA SE REALICE UNA CAMPAÑA EN MEDIOS DE COMUNICACIÓN Y ESTABLECIMIENTOS EDUCATIVOS PÚBLICOS Y PRIVADOS DE PREVENCIÓN Y CONCIENTIZACIÓN SOBRE LA VIOLENCIA EN ENTORNOS DIGITALES.</t>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA UNA CAMPAÑA MASIVA DE COMUNICACIÓN A TRAVÉS DE LOS MEDIOS DE COMUNICACIÓN Y EN LAS ESCUELAS PÚBLICAS Y PRIVADAS ORIENTADA A LA PREVENCIÓN Y CONCIENTIZACIÓN SOBRE EL "PHISHING".</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -4680,7 +4680,7 @@
         <v>2026</v>
       </c>
       <c r="B112" t="n">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -4689,12 +4689,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>S-68/26-PC</t>
+          <t>S-1254/25-PC</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA LA REALIZACION DE UNA CAMPAÑA DE COMUNICACIÓN ORIENTADA A LA PREVENCION Y CONCIENTIZACION DE LA LUDOPATIA INFANTIL, Y DE LA AUTODEPENDENCIA A DISPOSITIVOS MOVILES, VIDEOJUEGOS Y REDES SOCIALES EN MENORES DE 18 AÑOS.</t>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA SE REALICE UNA CAMPAÑA EN MEDIOS DE COMUNICACIÓN Y ESTABLECIMIENTOS EDUCATIVOS PÚBLICOS Y PRIVADOS DE PREVENCIÓN Y CONCIENTIZACIÓN SOBRE LA VIOLENCIA EN ENTORNOS DIGITALES.</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -4718,7 +4718,7 @@
         <v>2026</v>
       </c>
       <c r="B113" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -4727,12 +4727,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>S-881/26-PD</t>
+          <t>S-68/26-PC</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL QUINCUAGESIMO QUINTO ANIVERSARIO DEL PROGRAMA "FORMULA TUERCA Y TODOS LOS DEPORTES", EMITIDO POR LT4 RADIODIFUSORA MISIONES, PROV. HOMONIMA, EL 1° DE JULIO DE 2026.</t>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA LA REALIZACION DE UNA CAMPAÑA DE COMUNICACIÓN ORIENTADA A LA PREVENCION Y CONCIENTIZACION DE LA LUDOPATIA INFANTIL, Y DE LA AUTODEPENDENCIA A DISPOSITIVOS MOVILES, VIDEOJUEGOS Y REDES SOCIALES EN MENORES DE 18 AÑOS.</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -4756,34 +4756,72 @@
         <v>2026</v>
       </c>
       <c r="B114" t="n">
+        <v>406</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>S-881/26-PD</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL QUINCUAGESIMO QUINTO ANIVERSARIO DEL PROGRAMA "FORMULA TUERCA Y TODOS LOS DEPORTES", EMITIDO POR LT4 RADIODIFUSORA MISIONES, PROV. HOMONIMA, EL 1° DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B115" t="n">
         <v>407</v>
       </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
         <is>
           <t>PE-133/26-AC</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E115" t="inlineStr">
         <is>
           <t>MENSAJE N° 138/26 QUE SOLICITA ACUERDO PARA PROMOVER AL GRADO INMEDIATO SUPERIOR, AL 31 DE DICIEMBRE DE 2025, AL GENERAL DE BRIGADA SEBASTIAN IGNACIO IBAÑEZ.</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
+      <c r="F115" t="inlineStr">
         <is>
           <t>DE ACUERDOS -</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr">
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -5017,6 +5055,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I113" r:id="rId224"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId225"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId228"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática 2026-09-27 06:20 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -2134,7 +2134,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>DE ASUNTOS CONSTITUCIONALES -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES - DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática 2026-10-16 05:38 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4822,6 +4822,45 @@
         </is>
       </c>
       <c r="I115" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B116" t="n">
+        <v>408</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>PE-854/97-PL</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 1451/97 Y PROYECTO DE LEY APROBANDO EL TRATADO DE COOPERACION EN MATERIA DE PATENTES ( PCT ) ELABORADO EN WASHINGTON EL 19 DE JUNIO DE 1970 , ENMENDADO EL 28 DE SETIEMBRE DE 1979 Y MODIFICADO EL 3 DE FEBRERO DE 1984 Y EL REGLAMENTO DEL TRATADO DE COOPERACION EN MATERIA DE PATENTES
+( PCT</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>DE RELACIONES EXTERIORES Y CULTO - DE INDUSTRIA Y COMERCIO -</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -5057,6 +5096,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId230"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática 2026-10-22 05:55 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I116"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3763,7 +3763,7 @@
         <v>2026</v>
       </c>
       <c r="B88" t="n">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -3772,12 +3772,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>S-709/26-PD</t>
+          <t>S-2204/25-PD</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
+          <t>SCHNEIDER: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR LA PRESENTACION OFICIAL DE LA "BIENAL INTERNACIONAL DE ESCULTURA DEL CHACO EDICION 2026", A REALIZARSE EN LA CDAD. DE RESISTENCIA, PROV. DEL CHACO, EL 6 DE MARZO.</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3801,7 +3801,7 @@
         <v>2026</v>
       </c>
       <c r="B89" t="n">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -3810,12 +3810,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>S-735/26-PD</t>
+          <t>S-709/26-PD</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3839,7 +3839,7 @@
         <v>2026</v>
       </c>
       <c r="B90" t="n">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -3848,12 +3848,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>S-892/26-PD</t>
+          <t>S-735/26-PD</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
+          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3877,7 +3877,7 @@
         <v>2026</v>
       </c>
       <c r="B91" t="n">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -3886,12 +3886,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>S-900/26-PD</t>
+          <t>S-892/26-PD</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
+          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3915,7 +3915,7 @@
         <v>2026</v>
       </c>
       <c r="B92" t="n">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -3924,12 +3924,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>S-934/26-PD</t>
+          <t>S-900/26-PD</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3953,60 +3953,60 @@
         <v>2026</v>
       </c>
       <c r="B93" t="n">
+        <v>385</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>S-934/26-PD</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B94" t="n">
         <v>386</v>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
         <is>
           <t>S-2149/25-PD
 S-300/26-PD</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>CAPITANICH: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA BIENAL INTERNACIONAL DE ESCULTURAS DE CHACO 2026, A REALIZARSE EN LA CDAD. DE RESISTENCIA, DEL 11 AL 19 DE JULIO DE 2026.</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B94" t="n">
-        <v>387</v>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>S-935/26-PD</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4030,7 +4030,7 @@
         <v>2026</v>
       </c>
       <c r="B95" t="n">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -4039,12 +4039,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>S-1006/26-PD</t>
+          <t>S-935/26-PD</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4068,7 +4068,7 @@
         <v>2026</v>
       </c>
       <c r="B96" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -4077,12 +4077,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>S-1017/26-PD</t>
+          <t>S-1006/26-PD</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4106,7 +4106,7 @@
         <v>2026</v>
       </c>
       <c r="B97" t="n">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -4115,12 +4115,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>S-1020/26-PD</t>
+          <t>S-1017/26-PD</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
+          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4144,7 +4144,7 @@
         <v>2026</v>
       </c>
       <c r="B98" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -4153,12 +4153,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>S-1037/26-PD</t>
+          <t>S-1020/26-PD</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
+          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4182,7 +4182,7 @@
         <v>2026</v>
       </c>
       <c r="B99" t="n">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -4191,12 +4191,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>S-1038/26-PD</t>
+          <t>S-1037/26-PD</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4220,7 +4220,7 @@
         <v>2026</v>
       </c>
       <c r="B100" t="n">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>S-1104/26-PD</t>
+          <t>S-1038/26-PD</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
+          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4258,7 +4258,7 @@
         <v>2026</v>
       </c>
       <c r="B101" t="n">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -4267,12 +4267,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>S-1122/26-PD</t>
+          <t>S-1104/26-PD</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4296,7 +4296,7 @@
         <v>2026</v>
       </c>
       <c r="B102" t="n">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -4305,12 +4305,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>S-1029/26-PD</t>
+          <t>S-1122/26-PD</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4334,60 +4334,60 @@
         <v>2026</v>
       </c>
       <c r="B103" t="n">
+        <v>395</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>S-1029/26-PD</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B104" t="n">
         <v>396</v>
       </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
         <is>
           <t>S-1154/26-PD
 S-1166/26-PD</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E104" t="inlineStr">
         <is>
           <t>ATAUCHE: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES EL NUEVO ANIVERSARIO DEL EXODO JUJEÑO, EL 23 DE AGOSTO DE 2026.</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B104" t="n">
-        <v>397</v>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>S-1165/26-PD</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -4411,7 +4411,7 @@
         <v>2026</v>
       </c>
       <c r="B105" t="n">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -4420,17 +4420,17 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>S-1152/25-PD</t>
+          <t>S-1165/26-PD</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ATAUCHE: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA RADIAL "VIAJANDO POR ARGENTINA".</t>
+          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -4449,7 +4449,7 @@
         <v>2026</v>
       </c>
       <c r="B106" t="n">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -4458,12 +4458,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>S-1563/25-PD</t>
+          <t>S-1152/25-PD</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LOS PREMIOS PRISMA 2025, A REALIZARSE EN LA CDAD. DE POSADAS, PROV. DE MISIONES, EL 18 DE OCTUBRE.</t>
+          <t>ATAUCHE: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA RADIAL "VIAJANDO POR ARGENTINA".</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4487,7 +4487,7 @@
         <v>2026</v>
       </c>
       <c r="B107" t="n">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -4496,12 +4496,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>S-1647/25-PD</t>
+          <t>S-1563/25-PD</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>LEAVY: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA "SALTA ES UNA CANCION" QUE SE EMITE POR LA TELEVISION SALTEÑA DESDE 1997.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LOS PREMIOS PRISMA 2025, A REALIZARSE EN LA CDAD. DE POSADAS, PROV. DE MISIONES, EL 18 DE OCTUBRE.</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4525,143 +4525,143 @@
         <v>2026</v>
       </c>
       <c r="B108" t="n">
+        <v>400</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>S-1647/25-PD</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LEAVY: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA "SALTA ES UNA CANCION" QUE SE EMITE POR LA TELEVISION SALTEÑA DESDE 1997.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B109" t="n">
         <v>401</v>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
         <is>
           <t>S-931/25-PD
 S-998/26-PD</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>VISCHI: PROYECTO DE DECLARACIÓN QUE ADHIERE A LA CELEBRACIÓN DEL DIA DEL PERIODISTA, EL 7 DE JUNIO.</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B109" t="n">
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B110" t="n">
         <v>402</v>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>ANEXO</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D110" t="inlineStr">
         <is>
           <t>CD-3/26-PL
 S-909/26-PL</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E110" t="inlineStr">
         <is>
           <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA LEY 25.565, DE PRESUPUESTO GENERAL DE GASTOS DE LA ADM. NACIONAL PARA EL EJERCICIO 2002 SOBRE READECUACION DEL REGIMEN DE SUBSIDIOS A LOS CONSUMOS RESIDENCIALES DE GAS NATURAL EN ZONAS FRIAS, REGULARIZACION DE DEUDAS ELECTRICAS Y DEROGA LOS DECRETOS 277/2022 Y 929/2013.</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
+      <c r="F110" t="inlineStr">
         <is>
           <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B110" t="n">
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B111" t="n">
         <v>402</v>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
         <is>
           <t>CD-3/26-PL
 S-909/26-PL</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA LEY 25.565, DE PRESUPUESTO GENERAL DE GASTOS DE LA ADM. NACIONAL PARA EL EJERCICIO 2002 SOBRE READECUACION DEL REGIMEN DE SUBSIDIOS A LOS CONSUMOS RESIDENCIALES DE GAS NATURAL EN ZONAS FRIAS, REGULARIZACION DE DEUDAS ELECTRICAS Y DEROGA LOS DECRETOS 277/2022 Y 929/2013.</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F111" t="inlineStr">
         <is>
           <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES - DE PRESUPUESTO Y HACIENDA -</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B111" t="n">
-        <v>403</v>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>S-229/25-PC</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA UNA CAMPAÑA MASIVA DE COMUNICACIÓN A TRAVÉS DE LOS MEDIOS DE COMUNICACIÓN Y EN LAS ESCUELAS PÚBLICAS Y PRIVADAS ORIENTADA A LA PREVENCIÓN Y CONCIENTIZACIÓN SOBRE EL "PHISHING".</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -4680,7 +4680,7 @@
         <v>2026</v>
       </c>
       <c r="B112" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -4689,12 +4689,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>S-1254/25-PC</t>
+          <t>S-229/25-PC</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA SE REALICE UNA CAMPAÑA EN MEDIOS DE COMUNICACIÓN Y ESTABLECIMIENTOS EDUCATIVOS PÚBLICOS Y PRIVADOS DE PREVENCIÓN Y CONCIENTIZACIÓN SOBRE LA VIOLENCIA EN ENTORNOS DIGITALES.</t>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA UNA CAMPAÑA MASIVA DE COMUNICACIÓN A TRAVÉS DE LOS MEDIOS DE COMUNICACIÓN Y EN LAS ESCUELAS PÚBLICAS Y PRIVADAS ORIENTADA A LA PREVENCIÓN Y CONCIENTIZACIÓN SOBRE EL "PHISHING".</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -4718,7 +4718,7 @@
         <v>2026</v>
       </c>
       <c r="B113" t="n">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -4727,12 +4727,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>S-68/26-PC</t>
+          <t>S-1254/25-PC</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA LA REALIZACION DE UNA CAMPAÑA DE COMUNICACIÓN ORIENTADA A LA PREVENCION Y CONCIENTIZACION DE LA LUDOPATIA INFANTIL, Y DE LA AUTODEPENDENCIA A DISPOSITIVOS MOVILES, VIDEOJUEGOS Y REDES SOCIALES EN MENORES DE 18 AÑOS.</t>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA SE REALICE UNA CAMPAÑA EN MEDIOS DE COMUNICACIÓN Y ESTABLECIMIENTOS EDUCATIVOS PÚBLICOS Y PRIVADOS DE PREVENCIÓN Y CONCIENTIZACIÓN SOBRE LA VIOLENCIA EN ENTORNOS DIGITALES.</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -4756,7 +4756,7 @@
         <v>2026</v>
       </c>
       <c r="B114" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -4765,12 +4765,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>S-881/26-PD</t>
+          <t>S-68/26-PC</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>ARCE Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL QUINCUAGESIMO QUINTO ANIVERSARIO DEL PROGRAMA "FORMULA TUERCA Y TODOS LOS DEPORTES", EMITIDO POR LT4 RADIODIFUSORA MISIONES, PROV. HOMONIMA, EL 1° DE JULIO DE 2026.</t>
+          <t>LOSADA: PROYECTO DE COMUNICACIÓN QUE SOLICITA LA REALIZACION DE UNA CAMPAÑA DE COMUNICACIÓN ORIENTADA A LA PREVENCION Y CONCIENTIZACION DE LA LUDOPATIA INFANTIL, Y DE LA AUTODEPENDENCIA A DISPOSITIVOS MOVILES, VIDEOJUEGOS Y REDES SOCIALES EN MENORES DE 18 AÑOS.</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -4794,7 +4794,7 @@
         <v>2026</v>
       </c>
       <c r="B115" t="n">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -4803,17 +4803,17 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>PE-133/26-AC</t>
+          <t>S-881/26-PD</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>MENSAJE N° 138/26 QUE SOLICITA ACUERDO PARA PROMOVER AL GRADO INMEDIATO SUPERIOR, AL 31 DE DICIEMBRE DE 2025, AL GENERAL DE BRIGADA SEBASTIAN IGNACIO IBAÑEZ.</t>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL QUINCUAGESIMO QUINTO ANIVERSARIO DEL PROGRAMA "FORMULA TUERCA Y TODOS LOS DEPORTES", EMITIDO POR LT4 RADIODIFUSORA MISIONES, PROV. HOMONIMA, EL 1° DE JULIO DE 2026.</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>DE ACUERDOS -</t>
+          <t>DE SISTEMAS, MEDIOS DE COMUNICACIÓN Y LIBERTAD DE EXPRESIÓN -</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -4832,35 +4832,149 @@
         <v>2026</v>
       </c>
       <c r="B116" t="n">
+        <v>407</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>PE-133/26-AC</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 138/26 QUE SOLICITA ACUERDO PARA PROMOVER AL GRADO INMEDIATO SUPERIOR, AL 31 DE DICIEMBRE DE 2025, AL GENERAL DE BRIGADA SEBASTIAN IGNACIO IBAÑEZ.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS -</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B117" t="n">
         <v>408</v>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
         <is>
           <t>PE-854/97-PL</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="E117" t="inlineStr">
         <is>
           <t>MENSAJE N° 1451/97 Y PROYECTO DE LEY APROBANDO EL TRATADO DE COOPERACION EN MATERIA DE PATENTES ( PCT ) ELABORADO EN WASHINGTON EL 19 DE JUNIO DE 1970 , ENMENDADO EL 28 DE SETIEMBRE DE 1979 Y MODIFICADO EL 3 DE FEBRERO DE 1984 Y EL REGLAMENTO DEL TRATADO DE COOPERACION EN MATERIA DE PATENTES
 ( PCT</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr">
+      <c r="F117" t="inlineStr">
         <is>
           <t>DE RELACIONES EXTERIORES Y CULTO - DE INDUSTRIA Y COMERCIO -</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B118" t="n">
+        <v>409</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ANEXO</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>PE-99/26-PL</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 108/26 Y PROYECTO DE LEY SOBRE MODIFICACIONES A LA LEY NACIONAL DE SALUD MENTAL N° 26.657.</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>DE SALUD - DE LEGISLACIÓN GENERAL -</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B119" t="n">
+        <v>409</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>PE-99/26-PL</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 108/26 Y PROYECTO DE LEY SOBRE MODIFICACIONES A LA LEY NACIONAL DE SALUD MENTAL N° 26.657.</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>DE SALUD - DE LEGISLACIÓN GENERAL -</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -5098,6 +5212,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId228"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId229"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I117" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I119" r:id="rId236"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>